<commit_message>
coord transform for solid edge
</commit_message>
<xml_diff>
--- a/python/scripts/oracle_upload/sectors.xlsx
+++ b/python/scripts/oracle_upload/sectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="scS" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="396">
   <si>
     <t xml:space="preserve">Lsector=</t>
   </si>
@@ -511,6 +511,12 @@
     <t xml:space="preserve">15</t>
   </si>
   <si>
+    <t xml:space="preserve">BEGGSPEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENDGSPEC</t>
+  </si>
+  <si>
     <t xml:space="preserve">S21</t>
   </si>
   <si>
@@ -524,6 +530,12 @@
   </si>
   <si>
     <t xml:space="preserve">16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEGSPEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENDSPEC</t>
   </si>
   <si>
     <t xml:space="preserve">S22</t>
@@ -1539,8 +1551,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="7.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="71.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="60.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="31.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="5.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="4.28"/>
@@ -4073,7 +4085,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L1048576"/>
   <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.29"/>
@@ -4216,10 +4228,10 @@
         <v>56.1799475065617</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="K5" s="12"/>
       <c r="L5" s="1" t="n">
@@ -4228,7 +4240,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B6" s="38" t="s">
         <v>155</v>
@@ -4237,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E6" s="2" t="n">
         <f aca="false">F4</f>
@@ -4256,10 +4268,10 @@
         <v>323.375557742782</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="K6" s="12"/>
       <c r="L6" s="1" t="n">
@@ -4268,16 +4280,16 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E7" s="2" t="n">
         <f aca="false">F4</f>
@@ -4296,10 +4308,10 @@
         <v>323.375557742782</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="K7" s="12"/>
       <c r="L7" s="1" t="n">
@@ -4308,7 +4320,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B8" s="38" t="n">
         <v>10</v>
@@ -4317,7 +4329,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E8" s="2" t="n">
         <f aca="false">F6</f>
@@ -4336,10 +4348,10 @@
         <v>333.333333333333</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="K8" s="12"/>
       <c r="L8" s="1" t="n">
@@ -4348,7 +4360,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B9" s="38" t="n">
         <v>10</v>
@@ -4357,7 +4369,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E9" s="2" t="n">
         <f aca="false">F8</f>
@@ -4373,13 +4385,13 @@
       </c>
       <c r="H9" s="5" t="n">
         <f aca="false">G9/0.3048</f>
-        <v>333.333333333333</v>
+        <v>333.333333333334</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="K9" s="12"/>
       <c r="L9" s="1" t="n">
@@ -4388,7 +4400,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B10" s="38" t="n">
         <v>10</v>
@@ -4397,7 +4409,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E10" s="2" t="n">
         <f aca="false">F9</f>
@@ -4416,10 +4428,10 @@
         <v>333.333333333333</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="K10" s="12"/>
       <c r="L10" s="1" t="n">
@@ -4428,7 +4440,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B11" s="38" t="n">
         <v>10</v>
@@ -4437,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E11" s="2" t="n">
         <f aca="false">F10</f>
@@ -4453,13 +4465,13 @@
       </c>
       <c r="H11" s="5" t="n">
         <f aca="false">G11/0.3048</f>
-        <v>333.333333333334</v>
+        <v>333.333333333333</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="K11" s="12"/>
       <c r="L11" s="1" t="n">
@@ -4468,7 +4480,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B12" s="38" t="n">
         <v>10</v>
@@ -4477,7 +4489,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E12" s="2" t="n">
         <f aca="false">F11</f>
@@ -4496,10 +4508,10 @@
         <v>333.333333333333</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="K12" s="12"/>
       <c r="L12" s="1" t="n">
@@ -4508,7 +4520,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B13" s="38" t="n">
         <v>10</v>
@@ -4517,7 +4529,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E13" s="2" t="n">
         <f aca="false">F12</f>
@@ -4536,10 +4548,10 @@
         <v>333.333333333333</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="K13" s="12"/>
       <c r="L13" s="1" t="n">
@@ -4557,7 +4569,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E14" s="2" t="n">
         <f aca="false">F13</f>
@@ -4573,13 +4585,13 @@
       </c>
       <c r="H14" s="5" t="n">
         <f aca="false">G14/0.3048</f>
-        <v>333.333333333333</v>
+        <v>333.333333333334</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="K14" s="12"/>
       <c r="L14" s="1" t="n">
@@ -4597,7 +4609,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E15" s="2" t="n">
         <f aca="false">F14</f>
@@ -4616,10 +4628,10 @@
         <v>333.333333333333</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="K15" s="12"/>
       <c r="L15" s="1" t="n">
@@ -4637,7 +4649,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">F15</f>
@@ -4648,17 +4660,17 @@
       </c>
       <c r="G16" s="9" t="n">
         <f aca="false">F16-E16</f>
-        <v>104.112000000001</v>
+        <v>104.112</v>
       </c>
       <c r="H16" s="10" t="n">
         <f aca="false">G16/0.3048</f>
-        <v>341.574803149608</v>
+        <v>341.574803149607</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="J16" s="32" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="K16" s="12"/>
       <c r="L16" s="1" t="n">
@@ -4676,7 +4688,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>2.512</v>
@@ -4693,10 +4705,10 @@
         <v>569.255249343832</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="K17" s="41" t="s">
         <v>105</v>
@@ -4710,13 +4722,13 @@
         <v>101</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>2.512</v>
@@ -4733,10 +4745,10 @@
         <v>569.255249343832</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="K18" s="41"/>
       <c r="L18" s="1" t="n">
@@ -4745,7 +4757,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B19" s="38" t="n">
         <v>10</v>
@@ -4754,7 +4766,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E19" s="2" t="n">
         <f aca="false">F17</f>
@@ -4772,7 +4784,7 @@
         <v>90.2526246719161</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="K19" s="41"/>
       <c r="L19" s="1" t="n">
@@ -4781,7 +4793,7 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B20" s="38" t="n">
         <v>10</v>
@@ -4790,7 +4802,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E20" s="2" t="n">
         <f aca="false">F19</f>
@@ -4814,7 +4826,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B21" s="38" t="n">
         <v>10</v>
@@ -4823,7 +4835,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E21" s="2" t="n">
         <f aca="false">F20</f>
@@ -4847,7 +4859,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B22" s="38" t="n">
         <v>10</v>
@@ -4856,7 +4868,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E22" s="2" t="n">
         <f aca="false">F21</f>
@@ -4880,7 +4892,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B23" s="38" t="n">
         <v>10</v>
@@ -4889,7 +4901,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E23" s="2" t="n">
         <f aca="false">F22</f>
@@ -4913,7 +4925,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B24" s="38" t="n">
         <v>10</v>
@@ -4922,7 +4934,7 @@
         <v>1</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E24" s="2" t="n">
         <f aca="false">F23</f>
@@ -4946,7 +4958,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B25" s="38" t="n">
         <v>10</v>
@@ -4955,7 +4967,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E25" s="2" t="n">
         <f aca="false">F24</f>
@@ -4979,7 +4991,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B26" s="38" t="n">
         <v>10</v>
@@ -4988,7 +5000,7 @@
         <v>1</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E26" s="2" t="n">
         <f aca="false">F25</f>
@@ -5012,7 +5024,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B27" s="38" t="n">
         <v>10</v>
@@ -5021,7 +5033,7 @@
         <v>1</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E27" s="2" t="n">
         <f aca="false">F26</f>
@@ -5045,7 +5057,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B28" s="38" t="n">
         <v>10</v>
@@ -5054,7 +5066,7 @@
         <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E28" s="2" t="n">
         <f aca="false">F27</f>
@@ -5078,7 +5090,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B29" s="38" t="n">
         <v>10</v>
@@ -5087,7 +5099,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E29" s="2" t="n">
         <f aca="false">F28</f>
@@ -5111,7 +5123,7 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B30" s="38" t="n">
         <v>10</v>
@@ -5120,7 +5132,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E30" s="2" t="n">
         <f aca="false">F29</f>
@@ -5138,7 +5150,7 @@
         <v>110.597116141732</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="K30" s="41"/>
       <c r="L30" s="1" t="n">
@@ -5147,7 +5159,7 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B31" s="38" t="n">
         <v>10</v>
@@ -5156,7 +5168,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E31" s="2" t="n">
         <f aca="false">F30</f>
@@ -5174,7 +5186,7 @@
         <v>119.648897637795</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="K31" s="41"/>
       <c r="L31" s="1" t="n">
@@ -5183,7 +5195,7 @@
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B32" s="38" t="n">
         <v>10</v>
@@ -5192,7 +5204,7 @@
         <v>1</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E32" s="2" t="n">
         <f aca="false">F31</f>
@@ -5216,7 +5228,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B33" s="38" t="n">
         <v>10</v>
@@ -5225,7 +5237,7 @@
         <v>1</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E33" s="2" t="n">
         <f aca="false">F32</f>
@@ -5249,7 +5261,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B34" s="38" t="n">
         <v>10</v>
@@ -5258,7 +5270,7 @@
         <v>1</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E34" s="2" t="n">
         <f aca="false">F33</f>
@@ -5276,7 +5288,7 @@
         <v>154.361902887139</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="K34" s="41"/>
       <c r="L34" s="1" t="n">
@@ -5285,7 +5297,7 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B35" s="38" t="n">
         <v>10</v>
@@ -5294,7 +5306,7 @@
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E35" s="2" t="n">
         <f aca="false">F34</f>
@@ -5312,10 +5324,10 @@
         <v>52.2424770341206</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="K35" s="41"/>
       <c r="L35" s="1" t="n">
@@ -5324,7 +5336,7 @@
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B36" s="38" t="n">
         <v>10</v>
@@ -5333,7 +5345,7 @@
         <v>1</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E36" s="2" t="n">
         <f aca="false">F35</f>
@@ -5351,10 +5363,10 @@
         <v>101.919291338583</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="K36" s="41"/>
       <c r="L36" s="1" t="n">
@@ -5363,7 +5375,7 @@
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B37" s="38" t="n">
         <v>11</v>
@@ -5372,7 +5384,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>686.410331</v>
@@ -5389,10 +5401,10 @@
         <v>90.7672900262465</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="K37" s="41"/>
       <c r="L37" s="1" t="n">
@@ -5427,7 +5439,7 @@
         <v>799.368562992126</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>151</v>
@@ -5439,7 +5451,7 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B39" s="38" t="n">
         <v>12</v>
@@ -5448,7 +5460,7 @@
         <v>1</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>700.528</v>
@@ -5465,10 +5477,10 @@
         <v>192.040449475065</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="J39" s="31" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="K39" s="41"/>
       <c r="L39" s="1" t="n">
@@ -5477,7 +5489,7 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B40" s="40" t="n">
         <v>13</v>
@@ -5486,7 +5498,7 @@
         <v>1</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E40" s="9" t="n">
         <v>739.999999</v>
@@ -5503,10 +5515,10 @@
         <v>60.2390748031495</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="J40" s="32" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="K40" s="41"/>
       <c r="L40" s="1" t="n">
@@ -5580,6 +5592,7 @@
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K59" s="42"/>
     </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="K4:K16"/>
@@ -5614,7 +5627,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -5637,13 +5650,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>517.54</v>
@@ -5660,18 +5673,18 @@
         <v>8.02654855643056</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>519.986492</v>
@@ -5688,18 +5701,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>524.386492</v>
@@ -5716,18 +5729,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>528.786492</v>
@@ -5744,18 +5757,18 @@
         <v>14.435695538058</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>533.186492</v>
@@ -5772,18 +5785,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>537.586492</v>
@@ -5800,18 +5813,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>541.986492</v>
@@ -5828,18 +5841,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>546.386492</v>
@@ -5856,18 +5869,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>550.786492</v>
@@ -5884,18 +5897,18 @@
         <v>14.435695538058</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>555.186492</v>
@@ -5912,18 +5925,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>559.586492</v>
@@ -5940,7 +5953,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I12" s="1" t="n">
         <v>26</v>
@@ -5948,13 +5961,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>563.986492</v>
@@ -5971,7 +5984,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I13" s="1" t="n">
         <v>27</v>
@@ -5979,13 +5992,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>568.386492</v>
@@ -6002,7 +6015,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I14" s="1" t="n">
         <v>28</v>
@@ -6010,13 +6023,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>572.786492</v>
@@ -6033,7 +6046,7 @@
         <v>14.435695538058</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I15" s="1" t="n">
         <v>29</v>
@@ -6041,13 +6054,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>577.186492</v>
@@ -6064,7 +6077,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I16" s="1" t="n">
         <v>30</v>
@@ -6072,13 +6085,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>581.586492</v>
@@ -6095,7 +6108,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I17" s="1" t="n">
         <v>31</v>
@@ -6103,13 +6116,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>585.986492</v>
@@ -6126,7 +6139,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I18" s="1" t="n">
         <v>32</v>
@@ -6134,13 +6147,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>590.386492</v>
@@ -6157,7 +6170,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I19" s="1" t="n">
         <v>33</v>
@@ -6165,13 +6178,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>594.786492</v>
@@ -6188,7 +6201,7 @@
         <v>14.435695538058</v>
       </c>
       <c r="H20" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>34</v>
@@ -6196,13 +6209,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>599.186492</v>
@@ -6219,18 +6232,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>603.586492</v>
@@ -6247,7 +6260,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I22" s="1" t="n">
         <v>36</v>
@@ -6255,13 +6268,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>607.986492</v>
@@ -6278,7 +6291,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I23" s="1" t="n">
         <v>37</v>
@@ -6286,13 +6299,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>612.386492</v>
@@ -6309,7 +6322,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>38</v>
@@ -6317,13 +6330,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>616.786492</v>
@@ -6340,7 +6353,7 @@
         <v>14.435695538058</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I25" s="1" t="n">
         <v>39</v>
@@ -6348,13 +6361,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>621.186492</v>
@@ -6371,7 +6384,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I26" s="1" t="n">
         <v>40</v>
@@ -6379,13 +6392,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>625.586492</v>
@@ -6402,7 +6415,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I27" s="1" t="n">
         <v>41</v>
@@ -6410,13 +6423,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>629.986492</v>
@@ -6433,7 +6446,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I28" s="1" t="n">
         <v>42</v>
@@ -6441,13 +6454,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>634.386492</v>
@@ -6464,7 +6477,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I29" s="1" t="n">
         <v>43</v>
@@ -6472,13 +6485,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>638.786492</v>
@@ -6495,7 +6508,7 @@
         <v>14.435695538058</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I30" s="1" t="n">
         <v>44</v>
@@ -6503,13 +6516,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>643.186492</v>
@@ -6526,7 +6539,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I31" s="1" t="n">
         <v>45</v>
@@ -6534,13 +6547,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>647.586492</v>
@@ -6557,7 +6570,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I32" s="1" t="n">
         <v>46</v>
@@ -6565,13 +6578,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>651.986492</v>
@@ -6588,7 +6601,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I33" s="1" t="n">
         <v>47</v>
@@ -6596,13 +6609,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>656.386492</v>
@@ -6619,18 +6632,18 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>660.786492</v>
@@ -6647,18 +6660,18 @@
         <v>14.435695538058</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>665.186492</v>
@@ -6675,7 +6688,7 @@
         <v>14.4356955380577</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>
@@ -6704,7 +6717,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -6727,13 +6740,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>514.740001</v>
@@ -6750,7 +6763,7 @@
         <v>14.3295603674542</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I2" s="1" t="n">
         <v>13</v>
@@ -6758,13 +6771,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>519.107651</v>
@@ -6781,7 +6794,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>14</v>
@@ -6789,13 +6802,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>523.120318</v>
@@ -6812,7 +6825,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>15</v>
@@ -6820,13 +6833,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>527.132985</v>
@@ -6843,7 +6856,7 @@
         <v>13.164914698163</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I5" s="1" t="n">
         <v>16</v>
@@ -6851,13 +6864,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>531.145651</v>
@@ -6874,7 +6887,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I6" s="1" t="n">
         <v>17</v>
@@ -6882,13 +6895,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>535.158318</v>
@@ -6905,7 +6918,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I7" s="1" t="n">
         <v>18</v>
@@ -6913,13 +6926,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>539.170985</v>
@@ -6936,7 +6949,7 @@
         <v>13.164914698163</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I8" s="1" t="n">
         <v>19</v>
@@ -6944,13 +6957,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>543.183651</v>
@@ -6967,7 +6980,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I9" s="1" t="n">
         <v>20</v>
@@ -6975,13 +6988,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>547.196318</v>
@@ -6998,19 +7011,19 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>551.208985</v>
@@ -7027,7 +7040,7 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I11" s="1" t="n">
         <v>22</v>
@@ -7035,13 +7048,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>555.221651</v>
@@ -7058,7 +7071,7 @@
         <v>13.1649179790029</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I12" s="1" t="n">
         <v>23</v>
@@ -7066,13 +7079,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>559.234318</v>
@@ -7089,7 +7102,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I13" s="1" t="n">
         <v>24</v>
@@ -7097,13 +7110,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>563.246985</v>
@@ -7120,7 +7133,7 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I14" s="1" t="n">
         <v>25</v>
@@ -7128,13 +7141,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>567.259651</v>
@@ -7151,7 +7164,7 @@
         <v>13.1649179790029</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I15" s="1" t="n">
         <v>26</v>
@@ -7159,13 +7172,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>571.272318</v>
@@ -7182,7 +7195,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I16" s="1" t="n">
         <v>27</v>
@@ -7190,13 +7203,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>575.284985</v>
@@ -7213,19 +7226,19 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="I17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>579.297651</v>
@@ -7242,7 +7255,7 @@
         <v>13.1649179790029</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I18" s="1" t="n">
         <v>29</v>
@@ -7250,13 +7263,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>583.310318</v>
@@ -7273,7 +7286,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I19" s="1" t="n">
         <v>30</v>
@@ -7281,13 +7294,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>587.322985</v>
@@ -7304,7 +7317,7 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H20" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>31</v>
@@ -7312,13 +7325,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>591.335651</v>
@@ -7335,7 +7348,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I21" s="1" t="n">
         <v>32</v>
@@ -7343,13 +7356,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>595.348318</v>
@@ -7366,7 +7379,7 @@
         <v>13.1649179790029</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I22" s="1" t="n">
         <v>33</v>
@@ -7374,13 +7387,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>599.360985</v>
@@ -7397,7 +7410,7 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I23" s="1" t="n">
         <v>34</v>
@@ -7405,13 +7418,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>603.373651</v>
@@ -7428,7 +7441,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>35</v>
@@ -7436,13 +7449,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>607.386318</v>
@@ -7459,7 +7472,7 @@
         <v>13.1649179790029</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I25" s="1" t="n">
         <v>36</v>
@@ -7467,13 +7480,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>611.398985</v>
@@ -7490,7 +7503,7 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I26" s="1" t="n">
         <v>37</v>
@@ -7498,13 +7511,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>615.411651</v>
@@ -7521,7 +7534,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I27" s="1" t="n">
         <v>38</v>
@@ -7529,13 +7542,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>619.424318</v>
@@ -7552,7 +7565,7 @@
         <v>13.1649179790029</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I28" s="1" t="n">
         <v>39</v>
@@ -7560,13 +7573,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>623.436985</v>
@@ -7583,7 +7596,7 @@
         <v>13.1649146981626</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I29" s="1" t="n">
         <v>40</v>
@@ -7591,13 +7604,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>627.449651</v>
@@ -7614,7 +7627,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I30" s="1" t="n">
         <v>41</v>
@@ -7622,13 +7635,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>631.462318</v>
@@ -7645,7 +7658,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I31" s="1" t="n">
         <v>42</v>
@@ -7653,13 +7666,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>635.474985</v>
@@ -7676,7 +7689,7 @@
         <v>13.164914698163</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I32" s="1" t="n">
         <v>43</v>
@@ -7684,13 +7697,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>639.487651</v>
@@ -7707,7 +7720,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I33" s="1" t="n">
         <v>44</v>
@@ -7715,13 +7728,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>643.500318</v>
@@ -7738,7 +7751,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I34" s="1" t="n">
         <v>45</v>
@@ -7746,13 +7759,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>647.512985</v>
@@ -7769,7 +7782,7 @@
         <v>13.164914698163</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I35" s="1" t="n">
         <v>46</v>
@@ -7777,13 +7790,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>651.525651</v>
@@ -7800,7 +7813,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="I36" s="1" t="n">
         <v>47</v>
@@ -7808,13 +7821,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>655.538318</v>
@@ -7831,18 +7844,18 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="D38" s="2" t="n">
         <v>659.550985</v>
@@ -7859,18 +7872,18 @@
         <v>13.164914698163</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>663.563651</v>
@@ -7887,7 +7900,7 @@
         <v>13.1649179790025</v>
       </c>
       <c r="H39" s="0" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reconclile makeExcel.m with makeExcel.py
</commit_message>
<xml_diff>
--- a/python/scripts/oracle_upload/sectors.xlsx
+++ b/python/scripts/oracle_upload/sectors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AD_ACCEL\20240901s\RDB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AD_ACCEL\preRelease\RDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F009E48A-F2A8-436E-B63D-9BC608CC10BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589ED238-D39A-4F94-AB36-994F3D8894CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24165" yWindow="3735" windowWidth="17460" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9735" yWindow="405" windowWidth="15480" windowHeight="17175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scS" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="388">
   <si>
     <t>S00</t>
   </si>
@@ -1086,9 +1086,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>CLTH/BSYH1/BSYH2</t>
-  </si>
-  <si>
     <t>BEGL1</t>
   </si>
   <si>
@@ -1134,9 +1131,6 @@
     <t>BEGCLTH_1</t>
   </si>
   <si>
-    <t>ENDBSYH_2</t>
-  </si>
-  <si>
     <t>ENDUNDH</t>
   </si>
   <si>
@@ -1161,12 +1155,6 @@
     <t>ENDSFTH_2</t>
   </si>
   <si>
-    <t>BEGBSYA_1</t>
-  </si>
-  <si>
-    <t>ENDBSYA_2</t>
-  </si>
-  <si>
     <t>BEGL3</t>
   </si>
   <si>
@@ -1218,13 +1206,43 @@
     <t>HXRSS chicane</t>
   </si>
   <si>
-    <t>SXR extension</t>
-  </si>
-  <si>
     <t>SXRSS chicane</t>
   </si>
   <si>
-    <t>ENDBSY_2</t>
+    <t>ENDESA</t>
+  </si>
+  <si>
+    <t>BSYA</t>
+  </si>
+  <si>
+    <t>ESA</t>
+  </si>
+  <si>
+    <t>BRAM1B</t>
+  </si>
+  <si>
+    <t>ENDBSYA</t>
+  </si>
+  <si>
+    <t>CLTH/BSYH</t>
+  </si>
+  <si>
+    <t>ENDBSYH</t>
+  </si>
+  <si>
+    <t>partial cell</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>CBXFEL chicane #1</t>
+  </si>
+  <si>
+    <t>contains</t>
+  </si>
+  <si>
+    <t>Delta-II</t>
   </si>
 </sst>
 </file>
@@ -1410,9 +1428,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1421,6 +1436,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1705,7 +1723,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S61"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1804,7 +1822,7 @@
       <c r="I4" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="K4" s="24" t="s">
         <v>28</v>
       </c>
       <c r="L4" s="1">
@@ -1840,7 +1858,7 @@
         <f t="shared" ref="H5:H34" si="4">G5/0.3048</f>
         <v>333.33333333333331</v>
       </c>
-      <c r="K5" s="25"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="1">
         <v>2</v>
       </c>
@@ -1874,7 +1892,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333331</v>
       </c>
-      <c r="K6" s="25"/>
+      <c r="K6" s="24"/>
       <c r="L6" s="1">
         <v>3</v>
       </c>
@@ -1908,7 +1926,7 @@
         <f t="shared" si="4"/>
         <v>333.3333333333332</v>
       </c>
-      <c r="K7" s="25"/>
+      <c r="K7" s="24"/>
       <c r="L7" s="1">
         <v>4</v>
       </c>
@@ -1942,7 +1960,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333337</v>
       </c>
-      <c r="K8" s="25"/>
+      <c r="K8" s="24"/>
       <c r="L8" s="1">
         <v>5</v>
       </c>
@@ -1976,7 +1994,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333337</v>
       </c>
-      <c r="K9" s="25"/>
+      <c r="K9" s="24"/>
       <c r="L9" s="1">
         <v>6</v>
       </c>
@@ -2010,7 +2028,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333303</v>
       </c>
-      <c r="K10" s="25"/>
+      <c r="K10" s="24"/>
       <c r="L10" s="1">
         <v>7</v>
       </c>
@@ -2044,7 +2062,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333337</v>
       </c>
-      <c r="K11" s="25"/>
+      <c r="K11" s="24"/>
       <c r="L11" s="1">
         <v>8</v>
       </c>
@@ -2078,7 +2096,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333337</v>
       </c>
-      <c r="K12" s="25"/>
+      <c r="K12" s="24"/>
       <c r="L12" s="1">
         <v>9</v>
       </c>
@@ -2118,7 +2136,7 @@
       <c r="J13" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="K13" s="25"/>
+      <c r="K13" s="24"/>
       <c r="L13" s="1">
         <v>10</v>
       </c>
@@ -2158,7 +2176,7 @@
       <c r="J14" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="K14" s="25"/>
+      <c r="K14" s="24"/>
       <c r="L14" s="1">
         <v>11</v>
       </c>
@@ -2198,7 +2216,7 @@
       <c r="J15" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="K15" s="25"/>
+      <c r="K15" s="24"/>
       <c r="L15" s="1">
         <v>12</v>
       </c>
@@ -2238,7 +2256,7 @@
       <c r="J16" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="K16" s="25"/>
+      <c r="K16" s="24"/>
       <c r="L16" s="1">
         <v>13</v>
       </c>
@@ -2278,7 +2296,7 @@
       <c r="J17" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="K17" s="25"/>
+      <c r="K17" s="24"/>
       <c r="L17" s="1">
         <v>14</v>
       </c>
@@ -2318,7 +2336,7 @@
       <c r="J18" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="K18" s="25"/>
+      <c r="K18" s="24"/>
       <c r="L18" s="1">
         <v>15</v>
       </c>
@@ -2358,7 +2376,7 @@
       <c r="J19" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K19" s="25"/>
+      <c r="K19" s="24"/>
       <c r="L19" s="1">
         <v>16</v>
       </c>
@@ -2398,7 +2416,7 @@
       <c r="J20" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="K20" s="25"/>
+      <c r="K20" s="24"/>
       <c r="L20" s="1">
         <v>17</v>
       </c>
@@ -2438,7 +2456,7 @@
       <c r="J21" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="K21" s="25"/>
+      <c r="K21" s="24"/>
       <c r="L21" s="1">
         <v>18</v>
       </c>
@@ -2478,7 +2496,7 @@
       <c r="J22" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="K22" s="25"/>
+      <c r="K22" s="24"/>
       <c r="L22" s="1">
         <v>19</v>
       </c>
@@ -2518,7 +2536,7 @@
       <c r="J23" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="K23" s="25"/>
+      <c r="K23" s="24"/>
       <c r="L23" s="1">
         <v>20</v>
       </c>
@@ -2558,7 +2576,7 @@
       <c r="J24" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="K24" s="25"/>
+      <c r="K24" s="24"/>
       <c r="L24" s="1">
         <v>21</v>
       </c>
@@ -2598,7 +2616,7 @@
       <c r="J25" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="K25" s="25"/>
+      <c r="K25" s="24"/>
       <c r="L25" s="1">
         <v>22</v>
       </c>
@@ -2638,7 +2656,7 @@
       <c r="J26" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="K26" s="25"/>
+      <c r="K26" s="24"/>
       <c r="L26" s="1">
         <v>23</v>
       </c>
@@ -2678,7 +2696,7 @@
       <c r="J27" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="K27" s="25"/>
+      <c r="K27" s="24"/>
       <c r="L27" s="1">
         <v>24</v>
       </c>
@@ -2718,7 +2736,7 @@
       <c r="J28" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="K28" s="25"/>
+      <c r="K28" s="24"/>
       <c r="L28" s="1">
         <v>25</v>
       </c>
@@ -2758,7 +2776,7 @@
       <c r="J29" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="K29" s="25"/>
+      <c r="K29" s="24"/>
       <c r="L29" s="1">
         <v>26</v>
       </c>
@@ -2798,7 +2816,7 @@
       <c r="J30" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="K30" s="25"/>
+      <c r="K30" s="24"/>
       <c r="L30" s="1">
         <v>27</v>
       </c>
@@ -2838,7 +2856,7 @@
       <c r="J31" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="K31" s="25"/>
+      <c r="K31" s="24"/>
       <c r="L31" s="1">
         <v>28</v>
       </c>
@@ -2872,7 +2890,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333303</v>
       </c>
-      <c r="K32" s="25"/>
+      <c r="K32" s="24"/>
       <c r="L32" s="1">
         <v>29</v>
       </c>
@@ -2906,7 +2924,7 @@
         <f t="shared" si="4"/>
         <v>333.33333333333303</v>
       </c>
-      <c r="K33" s="25"/>
+      <c r="K33" s="24"/>
       <c r="L33" s="1">
         <v>30</v>
       </c>
@@ -2943,7 +2961,7 @@
       <c r="J34" s="18" t="s">
         <v>323</v>
       </c>
-      <c r="K34" s="26"/>
+      <c r="K34" s="25"/>
       <c r="L34" s="1">
         <v>31</v>
       </c>
@@ -2981,7 +2999,7 @@
       <c r="J35" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="K35" s="27" t="s">
+      <c r="K35" s="26" t="s">
         <v>29</v>
       </c>
       <c r="L35" s="1">
@@ -3019,7 +3037,7 @@
       <c r="I36" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K36" s="25"/>
+      <c r="K36" s="24"/>
       <c r="L36" s="1">
         <v>33</v>
       </c>
@@ -3052,7 +3070,7 @@
         <f t="shared" si="6"/>
         <v>85.171587926509247</v>
       </c>
-      <c r="K37" s="25"/>
+      <c r="K37" s="24"/>
       <c r="L37" s="1">
         <v>34</v>
       </c>
@@ -3085,7 +3103,7 @@
         <f t="shared" si="6"/>
         <v>90.504265091863431</v>
       </c>
-      <c r="K38" s="25"/>
+      <c r="K38" s="24"/>
       <c r="L38" s="1">
         <v>35</v>
       </c>
@@ -3118,7 +3136,7 @@
         <f t="shared" si="6"/>
         <v>100.17946194225736</v>
       </c>
-      <c r="K39" s="25"/>
+      <c r="K39" s="24"/>
       <c r="L39" s="1">
         <v>36</v>
       </c>
@@ -3151,7 +3169,7 @@
         <f t="shared" si="6"/>
         <v>89.236876640419837</v>
       </c>
-      <c r="K40" s="25"/>
+      <c r="K40" s="24"/>
       <c r="L40" s="1">
         <v>37</v>
       </c>
@@ -3184,7 +3202,7 @@
         <f t="shared" si="6"/>
         <v>90.484908136482858</v>
       </c>
-      <c r="K41" s="25"/>
+      <c r="K41" s="24"/>
       <c r="L41" s="1">
         <v>38</v>
       </c>
@@ -3217,7 +3235,7 @@
         <f t="shared" si="6"/>
         <v>75.762795275590648</v>
       </c>
-      <c r="K42" s="25"/>
+      <c r="K42" s="24"/>
       <c r="L42" s="1">
         <v>39</v>
       </c>
@@ -3250,7 +3268,7 @@
         <f t="shared" si="6"/>
         <v>95.227034120734857</v>
       </c>
-      <c r="K43" s="25"/>
+      <c r="K43" s="24"/>
       <c r="L43" s="1">
         <v>40</v>
       </c>
@@ -3283,7 +3301,7 @@
         <f t="shared" si="6"/>
         <v>99.886811023622172</v>
       </c>
-      <c r="K44" s="25"/>
+      <c r="K44" s="24"/>
       <c r="L44" s="1">
         <v>41</v>
       </c>
@@ -3316,7 +3334,7 @@
         <f t="shared" si="6"/>
         <v>88.113845144356958</v>
       </c>
-      <c r="K45" s="25"/>
+      <c r="K45" s="24"/>
       <c r="L45" s="1">
         <v>42</v>
       </c>
@@ -3349,7 +3367,7 @@
         <f t="shared" si="6"/>
         <v>95.997703412073378</v>
       </c>
-      <c r="K46" s="25"/>
+      <c r="K46" s="24"/>
       <c r="L46" s="1">
         <v>43</v>
       </c>
@@ -3385,7 +3403,7 @@
       <c r="J47" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="K47" s="25"/>
+      <c r="K47" s="24"/>
       <c r="L47" s="1">
         <v>44</v>
       </c>
@@ -3415,13 +3433,13 @@
         <v>41.929491999999982</v>
       </c>
       <c r="H48" s="3">
-        <f t="shared" ref="H48:H58" si="9">G48/0.3048</f>
+        <f t="shared" ref="H48:H57" si="9">G48/0.3048</f>
         <v>137.56395013123353</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="K48" s="25"/>
+        <v>339</v>
+      </c>
+      <c r="K48" s="24"/>
       <c r="L48" s="1">
         <v>45</v>
       </c>
@@ -3454,7 +3472,7 @@
         <f t="shared" si="9"/>
         <v>115.48556430446172</v>
       </c>
-      <c r="K49" s="25"/>
+      <c r="K49" s="24"/>
       <c r="L49" s="1">
         <v>46</v>
       </c>
@@ -3487,7 +3505,7 @@
         <f t="shared" si="9"/>
         <v>115.48556430446209</v>
       </c>
-      <c r="K50" s="25"/>
+      <c r="K50" s="24"/>
       <c r="L50" s="1">
         <v>47</v>
       </c>
@@ -3521,9 +3539,9 @@
         <v>132.8740157480315</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="K51" s="25"/>
+        <v>340</v>
+      </c>
+      <c r="K51" s="24"/>
       <c r="L51" s="1">
         <v>48</v>
       </c>
@@ -3557,12 +3575,12 @@
         <v>52.242480314960531</v>
       </c>
       <c r="I52" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="J52" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="J52" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="K52" s="25"/>
+      <c r="K52" s="24"/>
       <c r="L52" s="1">
         <v>49</v>
       </c>
@@ -3596,12 +3614,12 @@
         <v>101.91929133858285</v>
       </c>
       <c r="I53" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="J53" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="J53" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="K53" s="25"/>
+      <c r="K53" s="24"/>
       <c r="L53" s="1">
         <v>50</v>
       </c>
@@ -3634,12 +3652,12 @@
         <v>90.767290026246471</v>
       </c>
       <c r="I54" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="J54" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="J54" s="17" t="s">
-        <v>347</v>
-      </c>
-      <c r="K54" s="25"/>
+      <c r="K54" s="24"/>
       <c r="L54" s="1">
         <v>51</v>
       </c>
@@ -3655,7 +3673,7 @@
         <v>1</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="E55" s="3">
         <v>700.52800000000002</v>
@@ -3672,12 +3690,12 @@
         <v>130.42318241469803</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="J55" s="17" t="s">
-        <v>370</v>
-      </c>
-      <c r="K55" s="25"/>
+        <v>366</v>
+      </c>
+      <c r="K55" s="24"/>
       <c r="L55" s="1">
         <v>52</v>
       </c>
@@ -3693,7 +3711,7 @@
         <v>1</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="E56" s="3">
         <v>733.77200000000005</v>
@@ -3710,12 +3728,12 @@
         <v>73.253152887138924</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="J56" s="17" t="s">
-        <v>376</v>
-      </c>
-      <c r="K56" s="25"/>
+        <v>372</v>
+      </c>
+      <c r="K56" s="24"/>
       <c r="L56" s="1">
         <v>53</v>
       </c>
@@ -3731,7 +3749,7 @@
         <v>1</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="E57" s="1">
         <v>733.77200000000005</v>
@@ -3748,69 +3766,109 @@
         <v>80.439632545931474</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="J57" s="17" t="s">
-        <v>373</v>
-      </c>
-      <c r="K57" s="25"/>
+        <v>369</v>
+      </c>
+      <c r="K57" s="24"/>
       <c r="L57" s="1">
         <v>54</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="12" t="s">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B58" s="12">
+      <c r="B58" s="1">
         <v>9</v>
       </c>
-      <c r="C58" s="12">
-        <v>1</v>
-      </c>
-      <c r="D58" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="E58" s="12">
-        <v>176.02099999999999</v>
-      </c>
-      <c r="F58" s="13">
+      <c r="C58" s="1">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="E58" s="1">
+        <v>131.417</v>
+      </c>
+      <c r="F58" s="3">
         <v>313.05599999999998</v>
       </c>
-      <c r="G58" s="13">
+      <c r="G58" s="3">
         <f t="shared" si="8"/>
-        <v>137.035</v>
-      </c>
-      <c r="H58" s="14">
-        <f t="shared" si="9"/>
-        <v>449.58989501312334</v>
-      </c>
-      <c r="I58" s="12"/>
-      <c r="J58" s="18" t="s">
-        <v>381</v>
+        <v>181.63899999999998</v>
+      </c>
+      <c r="H58" s="2">
+        <f>G58/0.3048</f>
+        <v>595.92847769028867</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="J58" s="17" t="s">
+        <v>380</v>
       </c>
       <c r="K58" s="24"/>
       <c r="L58" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+    <row r="59" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="B59" s="12">
+        <v>9</v>
+      </c>
+      <c r="C59" s="12">
+        <v>1</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="E59" s="12">
+        <v>313.05599999999998</v>
+      </c>
+      <c r="F59" s="13">
+        <v>455.10700000000003</v>
+      </c>
+      <c r="G59" s="13">
+        <f t="shared" ref="G59" si="10">F59-E59</f>
+        <v>142.05100000000004</v>
+      </c>
+      <c r="H59" s="14">
+        <f t="shared" ref="H59" si="11">G59/0.3048</f>
+        <v>466.04658792650929</v>
+      </c>
+      <c r="I59" s="12" t="s">
+        <v>380</v>
+      </c>
+      <c r="J59" s="18" t="s">
+        <v>376</v>
+      </c>
+      <c r="K59" s="25"/>
+      <c r="L59" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
-        <v>1</v>
-      </c>
-      <c r="B61" s="20" t="s">
-        <v>338</v>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>1</v>
+      </c>
+      <c r="B62" s="20" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="K4:K34"/>
-    <mergeCell ref="K35:K57"/>
+    <mergeCell ref="K35:K59"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="61" orientation="portrait" r:id="rId1"/>
@@ -3822,7 +3880,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T56"/>
+  <dimension ref="A1:T55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
@@ -3926,12 +3984,12 @@
         <v>56.179947506561689</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="K4" s="25" t="s">
+        <v>347</v>
+      </c>
+      <c r="K4" s="24" t="s">
         <v>28</v>
       </c>
       <c r="L4" s="1">
@@ -3968,12 +4026,12 @@
         <v>323.37555774278189</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="K5" s="25"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="1">
         <v>2</v>
       </c>
@@ -4013,7 +4071,7 @@
       <c r="J6" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K6" s="25"/>
+      <c r="K6" s="24"/>
       <c r="L6" s="1">
         <v>3</v>
       </c>
@@ -4053,7 +4111,7 @@
       <c r="J7" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="K7" s="25"/>
+      <c r="K7" s="24"/>
       <c r="L7" s="1">
         <v>4</v>
       </c>
@@ -4091,9 +4149,9 @@
         <v>163</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="K8" s="25"/>
+        <v>336</v>
+      </c>
+      <c r="K8" s="24"/>
       <c r="L8" s="1">
         <v>5</v>
       </c>
@@ -4128,12 +4186,12 @@
         <v>333.33333333333451</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="K9" s="25"/>
+      <c r="K9" s="24"/>
       <c r="L9" s="1">
         <v>6</v>
       </c>
@@ -4173,7 +4231,7 @@
       <c r="J10" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="K10" s="25"/>
+      <c r="K10" s="24"/>
       <c r="L10" s="1">
         <v>7</v>
       </c>
@@ -4213,7 +4271,7 @@
       <c r="J11" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="K11" s="25"/>
+      <c r="K11" s="24"/>
       <c r="L11" s="1">
         <v>8</v>
       </c>
@@ -4253,7 +4311,7 @@
       <c r="J12" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="K12" s="25"/>
+      <c r="K12" s="24"/>
       <c r="L12" s="1">
         <v>9</v>
       </c>
@@ -4293,7 +4351,7 @@
       <c r="J13" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="K13" s="25"/>
+      <c r="K13" s="24"/>
       <c r="L13" s="1">
         <v>10</v>
       </c>
@@ -4330,9 +4388,9 @@
         <v>331</v>
       </c>
       <c r="J14" s="18" t="s">
-        <v>349</v>
-      </c>
-      <c r="K14" s="26"/>
+        <v>348</v>
+      </c>
+      <c r="K14" s="25"/>
       <c r="L14" s="1">
         <v>11</v>
       </c>
@@ -4348,7 +4406,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>335</v>
+        <v>381</v>
       </c>
       <c r="E15" s="3">
         <v>2.512</v>
@@ -4365,14 +4423,12 @@
         <v>569.25524934383191</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="K15" s="27" t="s">
-        <v>29</v>
-      </c>
+        <v>382</v>
+      </c>
+      <c r="K15" s="26"/>
       <c r="L15" s="1">
         <v>12</v>
       </c>
@@ -4408,7 +4464,7 @@
       <c r="I16" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K16" s="25"/>
+      <c r="K16" s="24"/>
       <c r="L16" s="1">
         <v>13</v>
       </c>
@@ -4441,7 +4497,7 @@
         <f t="shared" si="4"/>
         <v>91.041010498687683</v>
       </c>
-      <c r="K17" s="25"/>
+      <c r="K17" s="24"/>
       <c r="L17" s="1">
         <v>14</v>
       </c>
@@ -4474,7 +4530,7 @@
         <f t="shared" si="4"/>
         <v>95.802821522309742</v>
       </c>
-      <c r="K18" s="25"/>
+      <c r="K18" s="24"/>
       <c r="L18" s="1">
         <v>15</v>
       </c>
@@ -4507,7 +4563,7 @@
         <f t="shared" si="4"/>
         <v>86.220472440944789</v>
       </c>
-      <c r="K19" s="25"/>
+      <c r="K19" s="24"/>
       <c r="L19" s="1">
         <v>16</v>
       </c>
@@ -4540,7 +4596,7 @@
         <f t="shared" si="4"/>
         <v>91.108923884514368</v>
       </c>
-      <c r="K20" s="25"/>
+      <c r="K20" s="24"/>
       <c r="L20" s="1">
         <v>17</v>
       </c>
@@ -4573,7 +4629,7 @@
         <f t="shared" si="4"/>
         <v>91.010498687664068</v>
       </c>
-      <c r="K21" s="25"/>
+      <c r="K21" s="24"/>
       <c r="L21" s="1">
         <v>18</v>
       </c>
@@ -4606,7 +4662,7 @@
         <f t="shared" si="4"/>
         <v>95.636482939632657</v>
       </c>
-      <c r="K22" s="25"/>
+      <c r="K22" s="24"/>
       <c r="L22" s="1">
         <v>19</v>
       </c>
@@ -4639,7 +4695,7 @@
         <f t="shared" si="4"/>
         <v>86.417322834645589</v>
       </c>
-      <c r="K23" s="25"/>
+      <c r="K23" s="24"/>
       <c r="L23" s="1">
         <v>20</v>
       </c>
@@ -4672,7 +4728,7 @@
         <f t="shared" si="4"/>
         <v>91.108923884514368</v>
       </c>
-      <c r="K24" s="25"/>
+      <c r="K24" s="24"/>
       <c r="L24" s="1">
         <v>21</v>
       </c>
@@ -4705,7 +4761,7 @@
         <f t="shared" si="4"/>
         <v>91.043307086614163</v>
       </c>
-      <c r="K25" s="25"/>
+      <c r="K25" s="24"/>
       <c r="L25" s="1">
         <v>22</v>
       </c>
@@ -4738,7 +4794,7 @@
         <f t="shared" si="4"/>
         <v>91.043307086614163</v>
       </c>
-      <c r="K26" s="25"/>
+      <c r="K26" s="24"/>
       <c r="L26" s="1">
         <v>23</v>
       </c>
@@ -4774,7 +4830,7 @@
       <c r="J27" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="K27" s="25"/>
+      <c r="K27" s="24"/>
       <c r="L27" s="1">
         <v>24</v>
       </c>
@@ -4800,7 +4856,7 @@
         <v>551.20898499999998</v>
       </c>
       <c r="G28" s="3">
-        <f t="shared" ref="G28:G37" si="6">F28-E28</f>
+        <f t="shared" ref="G28:G36" si="6">F28-E28</f>
         <v>36.468983999999978</v>
       </c>
       <c r="H28" s="3">
@@ -4808,9 +4864,9 @@
         <v>119.6488976377952</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="K28" s="25"/>
+        <v>351</v>
+      </c>
+      <c r="K28" s="24"/>
       <c r="L28" s="1">
         <v>25</v>
       </c>
@@ -4843,7 +4899,7 @@
         <f>G29/0.3048</f>
         <v>118.48425196850404</v>
       </c>
-      <c r="K29" s="25"/>
+      <c r="K29" s="24"/>
       <c r="L29" s="1">
         <v>26</v>
       </c>
@@ -4876,7 +4932,7 @@
         <f>G30/0.3048</f>
         <v>118.48425196850404</v>
       </c>
-      <c r="K30" s="25"/>
+      <c r="K30" s="24"/>
       <c r="L30" s="1">
         <v>27</v>
       </c>
@@ -4910,9 +4966,9 @@
         <v>154.36190288713891</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="K31" s="25"/>
+        <v>350</v>
+      </c>
+      <c r="K31" s="24"/>
       <c r="L31" s="1">
         <v>28</v>
       </c>
@@ -4946,12 +5002,12 @@
         <v>52.24247703412064</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>355</v>
-      </c>
-      <c r="K32" s="25"/>
+        <v>353</v>
+      </c>
+      <c r="K32" s="24"/>
       <c r="L32" s="1">
         <v>29</v>
       </c>
@@ -4985,12 +5041,12 @@
         <v>101.91929133858285</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="K33" s="25"/>
+        <v>355</v>
+      </c>
+      <c r="K33" s="24"/>
       <c r="L33" s="1">
         <v>30</v>
       </c>
@@ -5023,147 +5079,112 @@
         <v>90.767290026246471</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="K34" s="25"/>
+        <v>357</v>
+      </c>
+      <c r="K34" s="24"/>
       <c r="L34" s="1">
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>328</v>
+        <v>112</v>
       </c>
       <c r="B35" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C35" s="1">
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>328</v>
+        <v>111</v>
       </c>
       <c r="E35" s="3">
-        <v>69.408164999999997</v>
+        <v>700.52800000000002</v>
       </c>
       <c r="F35" s="3">
-        <v>313.05570299999999</v>
+        <v>759.06192899999996</v>
       </c>
       <c r="G35" s="3">
-        <f t="shared" ref="G35:G36" si="9">F35-E35</f>
-        <v>243.647538</v>
+        <f t="shared" ref="G35" si="9">F35-E35</f>
+        <v>58.533928999999944</v>
       </c>
       <c r="H35" s="2">
-        <f t="shared" ref="H35:H36" si="10">G35/0.3048</f>
-        <v>799.36856299212593</v>
+        <f t="shared" ref="H35" si="10">G35/0.3048</f>
+        <v>192.04044947506543</v>
       </c>
       <c r="I35" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="J35" s="17" t="s">
         <v>360</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="K35" s="25"/>
+      <c r="K35" s="24"/>
       <c r="L35" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B36" s="1">
-        <v>12</v>
-      </c>
-      <c r="C36" s="1">
-        <v>1</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E36" s="3">
-        <v>700.52800000000002</v>
-      </c>
-      <c r="F36" s="3">
-        <v>759.06192899999996</v>
-      </c>
-      <c r="G36" s="3">
-        <f t="shared" si="9"/>
-        <v>58.533928999999944</v>
-      </c>
-      <c r="H36" s="2">
-        <f t="shared" si="10"/>
-        <v>192.04044947506543</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="B36" s="12">
+        <v>13</v>
+      </c>
+      <c r="C36" s="12">
+        <v>1</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="E36" s="13">
+        <v>739.999999</v>
+      </c>
+      <c r="F36" s="13">
+        <v>758.36086899999998</v>
+      </c>
+      <c r="G36" s="13">
+        <f t="shared" si="6"/>
+        <v>18.360869999999977</v>
+      </c>
+      <c r="H36" s="14">
+        <f t="shared" ref="H36" si="11">G36/0.3048</f>
+        <v>60.239074803149528</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="J36" s="18" t="s">
         <v>363</v>
-      </c>
-      <c r="J36" s="17" t="s">
-        <v>364</v>
       </c>
       <c r="K36" s="25"/>
       <c r="L36" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="B37" s="12">
-        <v>13</v>
-      </c>
-      <c r="C37" s="12">
-        <v>1</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>365</v>
-      </c>
-      <c r="E37" s="13">
-        <v>739.999999</v>
-      </c>
-      <c r="F37" s="13">
-        <v>758.36086899999998</v>
-      </c>
-      <c r="G37" s="13">
-        <f t="shared" si="6"/>
-        <v>18.360869999999977</v>
-      </c>
-      <c r="H37" s="14">
-        <f t="shared" ref="H37" si="11">G37/0.3048</f>
-        <v>60.239074803149528</v>
-      </c>
-      <c r="I37" s="12" t="s">
-        <v>366</v>
-      </c>
-      <c r="J37" s="18" t="s">
-        <v>367</v>
-      </c>
-      <c r="K37" s="26"/>
-      <c r="L37" s="1">
-        <v>34</v>
-      </c>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K37" s="11"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B38" s="1"/>
       <c r="K38" s="11"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="B39" s="1"/>
+      <c r="A39" s="1">
+        <v>1</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>337</v>
+      </c>
       <c r="K39" s="11"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
-        <v>1</v>
-      </c>
-      <c r="B40" s="20" t="s">
-        <v>338</v>
-      </c>
       <c r="K40" s="11"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -5210,14 +5231,11 @@
     </row>
     <row r="55" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K55" s="11"/>
-    </row>
-    <row r="56" spans="11:11" x14ac:dyDescent="0.25">
-      <c r="K56" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="K4:K14"/>
-    <mergeCell ref="K15:K37"/>
+    <mergeCell ref="K15:K36"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="60" orientation="portrait" r:id="rId1"/>
@@ -5235,7 +5253,7 @@
     <col min="4" max="5" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.140625" style="3"/>
     <col min="7" max="7" width="9.140625" style="2"/>
-    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5260,6 +5278,12 @@
       <c r="G1" s="14" t="s">
         <v>26</v>
       </c>
+      <c r="H1" s="27" t="s">
+        <v>386</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>384</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -5285,8 +5309,8 @@
         <f>F2/0.3048</f>
         <v>8.0265485564305603</v>
       </c>
-      <c r="H2" t="s">
-        <v>379</v>
+      <c r="I2" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -5313,8 +5337,8 @@
         <f t="shared" ref="G3:G36" si="1">F3/0.3048</f>
         <v>14.435695538057667</v>
       </c>
-      <c r="H3" t="s">
-        <v>379</v>
+      <c r="H3" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -5341,8 +5365,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H4" t="s">
-        <v>379</v>
+      <c r="H4" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -5369,8 +5393,8 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H5" t="s">
-        <v>379</v>
+      <c r="H5" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -5397,8 +5421,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H6" t="s">
-        <v>379</v>
+      <c r="H6" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,8 +5449,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H7" t="s">
-        <v>379</v>
+      <c r="H7" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -5453,8 +5477,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H8" t="s">
-        <v>379</v>
+      <c r="H8" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -5481,8 +5505,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H9" t="s">
-        <v>379</v>
+      <c r="H9" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -5509,8 +5533,8 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H10" t="s">
-        <v>379</v>
+      <c r="H10" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -5537,8 +5561,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H11" t="s">
-        <v>379</v>
+      <c r="H11" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -5565,11 +5589,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I12" s="1">
-        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -5596,11 +5617,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I13" s="1">
-        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -5627,11 +5645,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I14" s="1">
-        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -5658,11 +5673,8 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I15" s="1">
-        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -5689,14 +5701,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I16" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>303</v>
       </c>
@@ -5720,14 +5729,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I17" s="1">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>304</v>
       </c>
@@ -5751,14 +5757,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I18" s="1">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>311</v>
       </c>
@@ -5782,14 +5785,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I19" s="1">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>305</v>
       </c>
@@ -5813,14 +5813,11 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I20" s="1">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>306</v>
       </c>
@@ -5844,11 +5841,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H21" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H21" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>307</v>
       </c>
@@ -5872,14 +5869,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I22" s="1">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>308</v>
       </c>
@@ -5903,14 +5897,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I23" s="1">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>309</v>
       </c>
@@ -5934,14 +5925,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I24" s="1">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>310</v>
       </c>
@@ -5965,14 +5953,11 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I25" s="1">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>312</v>
       </c>
@@ -5996,14 +5981,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H26" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I26" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>313</v>
       </c>
@@ -6027,14 +6009,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I27" s="1">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>314</v>
       </c>
@@ -6058,14 +6037,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H28" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I28" s="1">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>315</v>
       </c>
@@ -6089,14 +6065,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I29" s="1">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>321</v>
       </c>
@@ -6120,14 +6093,11 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H30" t="s">
+      <c r="H30" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I30" s="1">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>316</v>
       </c>
@@ -6151,14 +6121,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I31" s="1">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>317</v>
       </c>
@@ -6182,11 +6149,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H32" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I32" s="1">
-        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -6213,11 +6177,8 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H33" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I33" s="1">
-        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -6244,8 +6205,11 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H34" s="1" t="s">
         <v>210</v>
+      </c>
+      <c r="I34" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -6272,7 +6236,7 @@
         <f t="shared" si="1"/>
         <v>14.43569553805804</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H35" s="1" t="s">
         <v>210</v>
       </c>
     </row>
@@ -6300,7 +6264,7 @@
         <f t="shared" si="1"/>
         <v>14.435695538057667</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H36" s="1" t="s">
         <v>210</v>
       </c>
     </row>
@@ -6317,7 +6281,7 @@
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6342,6 +6306,12 @@
       <c r="G1" s="14" t="s">
         <v>26</v>
       </c>
+      <c r="H1" s="27" t="s">
+        <v>386</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>384</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -6367,11 +6337,8 @@
         <f t="shared" ref="G2:G4" si="1">F2/0.3048</f>
         <v>14.329560367454153</v>
       </c>
-      <c r="H2" t="s">
-        <v>209</v>
-      </c>
-      <c r="I2" s="1">
-        <v>13</v>
+      <c r="H2" s="1" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -6398,11 +6365,8 @@
         <f t="shared" si="1"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I3" s="1">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -6429,11 +6393,8 @@
         <f t="shared" si="1"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I4" s="1">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -6460,11 +6421,8 @@
         <f>F5/0.3048</f>
         <v>13.164914698162995</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I5" s="1">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -6491,11 +6449,8 @@
         <f t="shared" ref="G6:G39" si="3">F6/0.3048</f>
         <v>13.164917979002508</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I6" s="1">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -6522,11 +6477,8 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I7" s="1">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -6553,11 +6505,8 @@
         <f t="shared" si="3"/>
         <v>13.164914698162995</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I8" s="1">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -6584,11 +6533,8 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I9" s="1">
-        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -6615,10 +6561,9 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H10" t="s">
-        <v>377</v>
-      </c>
-      <c r="I10" s="1"/>
+      <c r="H10" s="1" t="s">
+        <v>373</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -6644,11 +6589,8 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I11" s="1">
-        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -6675,11 +6617,8 @@
         <f t="shared" si="3"/>
         <v>13.164917979002881</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I12" s="1">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -6706,11 +6645,8 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I13" s="1">
-        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -6737,11 +6673,8 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I14" s="1">
-        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -6768,11 +6701,8 @@
         <f t="shared" si="3"/>
         <v>13.164917979002881</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="I15" s="1">
-        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -6799,14 +6729,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I16" s="1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>265</v>
       </c>
@@ -6830,12 +6757,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H17" t="s">
-        <v>378</v>
-      </c>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H17" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>266</v>
       </c>
@@ -6859,14 +6785,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002881</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I18" s="1">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>267</v>
       </c>
@@ -6890,14 +6813,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I19" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>268</v>
       </c>
@@ -6921,14 +6841,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I20" s="1">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>269</v>
       </c>
@@ -6952,14 +6869,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I21" s="1">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>270</v>
       </c>
@@ -6983,14 +6897,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002881</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I22" s="1">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>271</v>
       </c>
@@ -7014,14 +6925,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I23" s="1">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>272</v>
       </c>
@@ -7045,14 +6953,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I24" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>273</v>
       </c>
@@ -7076,14 +6981,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002881</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I25" s="1">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>274</v>
       </c>
@@ -7107,14 +7009,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H26" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I26" s="1">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>275</v>
       </c>
@@ -7138,14 +7037,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I27" s="1">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>276</v>
       </c>
@@ -7169,14 +7065,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002881</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H28" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I28" s="1">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>277</v>
       </c>
@@ -7200,14 +7093,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162622</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I29" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>278</v>
       </c>
@@ -7231,14 +7121,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H30" t="s">
+      <c r="H30" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I30" s="1">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>279</v>
       </c>
@@ -7262,14 +7149,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I31" s="1">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>280</v>
       </c>
@@ -7293,14 +7177,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162995</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H32" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I32" s="1">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>281</v>
       </c>
@@ -7324,14 +7205,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H33" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I33" s="1">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>282</v>
       </c>
@@ -7355,14 +7233,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H34" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I34" s="1">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>283</v>
       </c>
@@ -7386,14 +7261,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162995</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H35" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I35" s="1">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>284</v>
       </c>
@@ -7417,14 +7289,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H36" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="I36" s="1">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>285</v>
       </c>
@@ -7448,11 +7317,11 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H37" t="s">
+      <c r="H37" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>286</v>
       </c>
@@ -7476,11 +7345,11 @@
         <f t="shared" si="3"/>
         <v>13.164914698162995</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H38" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>287</v>
       </c>
@@ -7504,7 +7373,7 @@
         <f t="shared" si="3"/>
         <v>13.164917979002508</v>
       </c>
-      <c r="H39" t="s">
+      <c r="H39" s="1" t="s">
         <v>210</v>
       </c>
     </row>

</xml_diff>